<commit_message>
updated so that it can take in upper case column names'
</commit_message>
<xml_diff>
--- a/results/tables.xlsx
+++ b/results/tables.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C51"/>
+  <dimension ref="A1:C17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -451,11 +451,11 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>USER_032</t>
+          <t>Jonathan C_20260116_171814</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>38.61</v>
+        <v>42.17</v>
       </c>
     </row>
     <row r="3">
@@ -464,11 +464,11 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>USER_045</t>
+          <t>Ben DeGioia_20260116_172416</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>40.57</v>
+        <v>43.86</v>
       </c>
     </row>
     <row r="4">
@@ -477,11 +477,11 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>USER_037</t>
+          <t>Chinenye Victoria Onukaogu_20260116_171323</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>41.9</v>
+        <v>44.22</v>
       </c>
     </row>
     <row r="5">
@@ -490,11 +490,11 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>USER_004</t>
+          <t>KP Ko_20260116_214646</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>42.17</v>
+        <v>47.78</v>
       </c>
     </row>
     <row r="6">
@@ -503,11 +503,11 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>USER_006</t>
+          <t>Nora_20260117_082206</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>43.86</v>
+        <v>48.58</v>
       </c>
     </row>
     <row r="7">
@@ -516,11 +516,11 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>USER_018</t>
+          <t>Catherine Meng_20260116_165524</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>43.86</v>
+        <v>49.47</v>
       </c>
     </row>
     <row r="8">
@@ -529,11 +529,11 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>USER_022</t>
+          <t>Haydn_20260117_104416</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>44.04</v>
+        <v>49.56</v>
       </c>
     </row>
     <row r="9">
@@ -542,11 +542,11 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>USER_048</t>
+          <t>Joanna Park_20260117_103454</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>44.04</v>
+        <v>50.53</v>
       </c>
     </row>
     <row r="10">
@@ -555,11 +555,11 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>USER_003</t>
+          <t>Helen Yoon_20260116_172314</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>44.22</v>
+        <v>51.33</v>
       </c>
     </row>
     <row r="11">
@@ -568,11 +568,11 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>USER_035</t>
+          <t>Tiffany Zhong_20260117_003118</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>44.48</v>
+        <v>51.78</v>
       </c>
     </row>
     <row r="12">
@@ -581,11 +581,11 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>USER_019</t>
+          <t>Grace Lee_20260117_114907</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>44.75</v>
+        <v>52.05</v>
       </c>
     </row>
     <row r="13">
@@ -594,11 +594,11 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>USER_028</t>
+          <t>Vianca Yoon_20260116_193608</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>45.73</v>
+        <v>53.2</v>
       </c>
     </row>
     <row r="14">
@@ -607,11 +607,11 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>USER_024</t>
+          <t>James Ahn_20260116_163855</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>47.69</v>
+        <v>53.38</v>
       </c>
     </row>
     <row r="15">
@@ -620,11 +620,11 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>USER_009</t>
+          <t>Jeremy Vinarao_20260117_055638</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>47.78</v>
+        <v>54</v>
       </c>
     </row>
     <row r="16">
@@ -633,11 +633,11 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>USER_029</t>
+          <t>Daniel Choi_20260116_184114</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>47.86</v>
+        <v>55.34</v>
       </c>
     </row>
     <row r="17">
@@ -646,453 +646,11 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>USER_013</t>
+          <t>Zoe Liao_20260116_231803</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>48.58</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="n">
-        <v>5</v>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>USER_040</t>
-        </is>
-      </c>
-      <c r="C18" t="n">
-        <v>48.67</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="n">
-        <v>5</v>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>USER_039</t>
-        </is>
-      </c>
-      <c r="C19" t="n">
-        <v>49.29</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="n">
-        <v>5</v>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>USER_002</t>
-        </is>
-      </c>
-      <c r="C20" t="n">
-        <v>49.47</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="n">
-        <v>5</v>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>USER_015</t>
-        </is>
-      </c>
-      <c r="C21" t="n">
-        <v>49.56</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="n">
-        <v>6</v>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>USER_014</t>
-        </is>
-      </c>
-      <c r="C22" t="n">
-        <v>50.53</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="n">
-        <v>6</v>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>USER_020</t>
-        </is>
-      </c>
-      <c r="C23" t="n">
-        <v>50.89</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="n">
-        <v>6</v>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>USER_033</t>
-        </is>
-      </c>
-      <c r="C24" t="n">
-        <v>50.98</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="n">
-        <v>6</v>
-      </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>USER_005</t>
-        </is>
-      </c>
-      <c r="C25" t="n">
-        <v>51.33</v>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="n">
-        <v>7</v>
-      </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>USER_044</t>
-        </is>
-      </c>
-      <c r="C26" t="n">
-        <v>51.42</v>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="n">
-        <v>7</v>
-      </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>USER_021</t>
-        </is>
-      </c>
-      <c r="C27" t="n">
-        <v>51.51</v>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="n">
-        <v>7</v>
-      </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>USER_011</t>
-        </is>
-      </c>
-      <c r="C28" t="n">
-        <v>51.78</v>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="n">
-        <v>7</v>
-      </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>USER_050</t>
-        </is>
-      </c>
-      <c r="C29" t="n">
-        <v>51.87</v>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="n">
-        <v>8</v>
-      </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>USER_016</t>
-        </is>
-      </c>
-      <c r="C30" t="n">
-        <v>52.05</v>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="n">
-        <v>8</v>
-      </c>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>USER_023</t>
-        </is>
-      </c>
-      <c r="C31" t="n">
-        <v>52.05</v>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="n">
-        <v>8</v>
-      </c>
-      <c r="B32" t="inlineStr">
-        <is>
-          <t>USER_026</t>
-        </is>
-      </c>
-      <c r="C32" t="n">
-        <v>52.22</v>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="n">
-        <v>8</v>
-      </c>
-      <c r="B33" t="inlineStr">
-        <is>
-          <t>USER_027</t>
-        </is>
-      </c>
-      <c r="C33" t="n">
-        <v>52.58</v>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="n">
-        <v>9</v>
-      </c>
-      <c r="B34" t="inlineStr">
-        <is>
-          <t>USER_008</t>
-        </is>
-      </c>
-      <c r="C34" t="n">
-        <v>53.2</v>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="n">
-        <v>9</v>
-      </c>
-      <c r="B35" t="inlineStr">
-        <is>
-          <t>USER_001</t>
-        </is>
-      </c>
-      <c r="C35" t="n">
-        <v>53.38</v>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="n">
-        <v>9</v>
-      </c>
-      <c r="B36" t="inlineStr">
-        <is>
-          <t>USER_042</t>
-        </is>
-      </c>
-      <c r="C36" t="n">
-        <v>53.47</v>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="n">
-        <v>9</v>
-      </c>
-      <c r="B37" t="inlineStr">
-        <is>
-          <t>USER_043</t>
-        </is>
-      </c>
-      <c r="C37" t="n">
-        <v>53.56</v>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" t="n">
-        <v>10</v>
-      </c>
-      <c r="B38" t="inlineStr">
-        <is>
-          <t>USER_047</t>
-        </is>
-      </c>
-      <c r="C38" t="n">
-        <v>53.56</v>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" t="n">
-        <v>10</v>
-      </c>
-      <c r="B39" t="inlineStr">
-        <is>
-          <t>USER_012</t>
-        </is>
-      </c>
-      <c r="C39" t="n">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" t="n">
-        <v>10</v>
-      </c>
-      <c r="B40" t="inlineStr">
-        <is>
-          <t>USER_046</t>
-        </is>
-      </c>
-      <c r="C40" t="n">
-        <v>54.27</v>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" t="n">
-        <v>10</v>
-      </c>
-      <c r="B41" t="inlineStr">
-        <is>
-          <t>USER_049</t>
-        </is>
-      </c>
-      <c r="C41" t="n">
-        <v>54.27</v>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" t="n">
-        <v>11</v>
-      </c>
-      <c r="B42" t="inlineStr">
-        <is>
-          <t>USER_025</t>
-        </is>
-      </c>
-      <c r="C42" t="n">
-        <v>54.54</v>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" t="n">
-        <v>11</v>
-      </c>
-      <c r="B43" t="inlineStr">
-        <is>
-          <t>USER_031</t>
-        </is>
-      </c>
-      <c r="C43" t="n">
-        <v>55.07</v>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" t="n">
-        <v>11</v>
-      </c>
-      <c r="B44" t="inlineStr">
-        <is>
-          <t>USER_036</t>
-        </is>
-      </c>
-      <c r="C44" t="n">
-        <v>55.16</v>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" t="n">
-        <v>11</v>
-      </c>
-      <c r="B45" t="inlineStr">
-        <is>
-          <t>USER_007</t>
-        </is>
-      </c>
-      <c r="C45" t="n">
-        <v>55.34</v>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" t="n">
-        <v>12</v>
-      </c>
-      <c r="B46" t="inlineStr">
-        <is>
-          <t>USER_017</t>
-        </is>
-      </c>
-      <c r="C46" t="n">
-        <v>55.69</v>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" t="n">
-        <v>12</v>
-      </c>
-      <c r="B47" t="inlineStr">
-        <is>
-          <t>USER_034</t>
-        </is>
-      </c>
-      <c r="C47" t="n">
-        <v>56.14</v>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" t="n">
-        <v>12</v>
-      </c>
-      <c r="B48" t="inlineStr">
-        <is>
-          <t>USER_041</t>
-        </is>
-      </c>
-      <c r="C48" t="n">
-        <v>56.14</v>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" t="n">
-        <v>12</v>
-      </c>
-      <c r="B49" t="inlineStr">
-        <is>
-          <t>USER_010</t>
-        </is>
-      </c>
-      <c r="C49" t="n">
         <v>56.94</v>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" t="n">
-        <v>12</v>
-      </c>
-      <c r="B50" t="inlineStr">
-        <is>
-          <t>USER_030</t>
-        </is>
-      </c>
-      <c r="C50" t="n">
-        <v>57.3</v>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" t="n">
-        <v>12</v>
-      </c>
-      <c r="B51" t="inlineStr">
-        <is>
-          <t>USER_038</t>
-        </is>
-      </c>
-      <c r="C51" t="n">
-        <v>61.12</v>
       </c>
     </row>
   </sheetData>

</xml_diff>